<commit_message>
Merge all projects into one solution and fix forms balsaab2
</commit_message>
<xml_diff>
--- a/ClinicVets/Data/ClinicVetsData.xlsx
+++ b/ClinicVets/Data/ClinicVetsData.xlsx
@@ -163,6 +163,38 @@
         </x:is>
       </x:c>
     </x:row>
+    <x:row r="3">
+      <x:c r="B3" t="inlineStr">
+        <x:is>
+          <x:t>balsam</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="C3" t="inlineStr">
+        <x:is>
+          <x:t>Balsam1!</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="A3" t="inlineStr">
+        <x:is>
+          <x:t>1234</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D3" t="inlineStr">
+        <x:is>
+          <x:t>balsam@gmail.com</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="E3" t="inlineStr">
+        <x:is>
+          <x:t>123456789</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F3" t="inlineStr">
+        <x:is>
+          <x:t>Secretary</x:t>
+        </x:is>
+      </x:c>
+    </x:row>
   </x:sheetData>
 </x:worksheet>
 </file>
</xml_diff>